<commit_message>
Rerun closed aggregate zero shot
</commit_message>
<xml_diff>
--- a/results/closed_aggregate_zero_shot_final/ilsp__Llama-Krikri-8B-Instruct-v1.5/closed_zero_shot_final.xlsx
+++ b/results/closed_aggregate_zero_shot_final/ilsp__Llama-Krikri-8B-Instruct-v1.5/closed_zero_shot_final.xlsx
@@ -478,10 +478,10 @@
         <v>52</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5961538461538461</v>
+        <v>0.5576923076923077</v>
       </c>
       <c r="F2" t="n">
-        <v>0.06870717031248968</v>
+        <v>0.06954637296657958</v>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
@@ -538,10 +538,10 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0.4534883720930232</v>
+        <v>0.4651162790697674</v>
       </c>
       <c r="H4" t="n">
-        <v>0.05399745837912383</v>
+        <v>0.05410046493374882</v>
       </c>
       <c r="I4" t="inlineStr"/>
     </row>
@@ -594,10 +594,10 @@
         <v>20</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0917662935482247</v>
+        <v>0.09933992677987828</v>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
@@ -652,10 +652,10 @@
         <v>35</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9142857142857143</v>
+        <v>0.9428571428571428</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04800960288096035</v>
+        <v>0.03980745977252778</v>
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
@@ -681,10 +681,10 @@
         <v>35</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="F9" t="n">
-        <v>0.08486978939800066</v>
+        <v>0.08140424227436861</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
@@ -713,7 +713,7 @@
         <v>0.3939393939393939</v>
       </c>
       <c r="F10" t="n">
-        <v>0.06060606060606062</v>
+        <v>0.06060606060606063</v>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
@@ -739,10 +739,10 @@
         <v>37</v>
       </c>
       <c r="E11" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.5675675675675675</v>
       </c>
       <c r="F11" t="n">
-        <v>0.08305895907471073</v>
+        <v>0.08256893144064577</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
@@ -768,16 +768,16 @@
         <v>451</v>
       </c>
       <c r="E12" t="n">
-        <v>0.589041095890411</v>
+        <v>0.5945205479452055</v>
       </c>
       <c r="F12" t="n">
-        <v>0.02495360435382393</v>
+        <v>0.02483097768976167</v>
       </c>
       <c r="G12" t="n">
-        <v>0.4534883720930232</v>
+        <v>0.4651162790697674</v>
       </c>
       <c r="H12" t="n">
-        <v>0.05399745837912383</v>
+        <v>0.05410046493374882</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>

</xml_diff>